<commit_message>
Atualização automática de preços de eletricidade
</commit_message>
<xml_diff>
--- a/output/spot_price_dailyHour_PT.xlsx
+++ b/output/spot_price_dailyHour_PT.xlsx
@@ -647,82 +647,82 @@
     </row>
     <row r="2">
       <c r="A2" s="3" t="n">
-        <v>46076</v>
+        <v>46077</v>
       </c>
       <c r="B2" t="n">
-        <v>23.89</v>
+        <v>28.23</v>
       </c>
       <c r="C2" t="n">
-        <v>19.91</v>
+        <v>23.4</v>
       </c>
       <c r="D2" t="n">
-        <v>18.24</v>
+        <v>21.3</v>
       </c>
       <c r="E2" t="n">
-        <v>12.63</v>
+        <v>20.29</v>
       </c>
       <c r="F2" t="n">
-        <v>10.58</v>
+        <v>18.87</v>
       </c>
       <c r="G2" t="n">
-        <v>18.03</v>
+        <v>21.31</v>
       </c>
       <c r="H2" t="n">
-        <v>24.23</v>
+        <v>21.31</v>
       </c>
       <c r="I2" t="n">
-        <v>35.02</v>
+        <v>23.52</v>
       </c>
       <c r="J2" t="n">
-        <v>35.49</v>
+        <v>26.04</v>
       </c>
       <c r="K2" t="n">
-        <v>14.52</v>
+        <v>15.82</v>
       </c>
       <c r="L2" t="n">
-        <v>10.54</v>
+        <v>2.38</v>
       </c>
       <c r="M2" t="n">
-        <v>10</v>
+        <v>0.65</v>
       </c>
       <c r="N2" t="n">
-        <v>9.99</v>
+        <v>0.58</v>
       </c>
       <c r="O2" t="n">
-        <v>9.039999999999999</v>
+        <v>0.26</v>
       </c>
       <c r="P2" t="n">
-        <v>8.24</v>
+        <v>0.15</v>
       </c>
       <c r="Q2" t="n">
-        <v>10</v>
+        <v>0.38</v>
       </c>
       <c r="R2" t="n">
-        <v>13.9</v>
+        <v>0.6</v>
       </c>
       <c r="S2" t="n">
-        <v>22.03</v>
+        <v>13.63</v>
       </c>
       <c r="T2" t="n">
-        <v>37.29</v>
+        <v>22.86</v>
       </c>
       <c r="U2" t="n">
-        <v>93.01000000000001</v>
+        <v>27.09</v>
       </c>
       <c r="V2" t="n">
-        <v>175.13</v>
+        <v>41.03</v>
       </c>
       <c r="W2" t="n">
-        <v>110.76</v>
+        <v>32.84</v>
       </c>
       <c r="X2" t="n">
-        <v>54.16</v>
+        <v>27.89</v>
       </c>
       <c r="Y2" t="n">
-        <v>31.38</v>
+        <v>25.39</v>
       </c>
       <c r="Z2" t="n">
-        <v>33.67</v>
+        <v>17.33</v>
       </c>
       <c r="AA2" t="inlineStr">
         <is>
@@ -730,7 +730,7 @@
         </is>
       </c>
       <c r="AB2" t="n">
-        <v>92.86</v>
+        <v>31.79</v>
       </c>
       <c r="AC2" t="inlineStr">
         <is>
@@ -738,19 +738,19 @@
         </is>
       </c>
       <c r="AD2" t="n">
-        <v>142.94</v>
+        <v>36.94</v>
       </c>
       <c r="AE2" t="inlineStr">
         <is>
-          <t>18h-20h</t>
+          <t>22h-24h</t>
         </is>
       </c>
       <c r="AF2" t="n">
-        <v>65.15000000000001</v>
+        <v>26.64</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
-          <t>0h-23h</t>
+          <t>9h-17h</t>
         </is>
       </c>
     </row>

</xml_diff>